<commit_message>
010: updated the routine file for today.
</commit_message>
<xml_diff>
--- a/data/daily_routine.xlsx
+++ b/data/daily_routine.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sai Swaroop\Desktop\Career\Learnings\AAA\projects\agents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sai Swaroop\Desktop\Innvt\APPS\Routine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F7212BA-4BE4-4A9B-AB23-0600A187FDE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322E2A70-A642-4206-8BED-4A91E72A33D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2DFCF397-A81A-4053-A0B6-07FE7B9B6438}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="61">
   <si>
     <t>23:40 – 07:00</t>
   </si>
@@ -127,9 +127,6 @@
   </si>
   <si>
     <t>woke up late</t>
-  </si>
-  <si>
-    <t>wake 5mins up before time</t>
   </si>
   <si>
     <t>started integration with telegram</t>
@@ -207,26 +204,17 @@
 (1-5)</t>
   </si>
   <si>
-    <t>good control over the ride</t>
-  </si>
-  <si>
-    <t>ride well</t>
-  </si>
-  <si>
-    <t>not able to focus as I am not 
-interested in the work</t>
-  </si>
-  <si>
-    <t>to focus more and learn something</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>not using time as planned</t>
-  </si>
-  <si>
-    <t>to spend the time as planned</t>
+    <t>working on learning Agentic AI</t>
+  </si>
+  <si>
+    <t>less focus</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>wake 5mins up before time and 
+hydrate well</t>
   </si>
 </sst>
 </file>
@@ -666,16 +654,16 @@
         <v>29</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>27</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>28</v>
@@ -701,16 +689,16 @@
         <v>3.5</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H2" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I2" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>23</v>
       </c>
@@ -718,10 +706,10 @@
         <v>30</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="D3" s="1">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E3" s="1">
         <v>2.5</v>
@@ -735,8 +723,8 @@
       <c r="H3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>34</v>
+      <c r="I3" s="6" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -747,10 +735,10 @@
         <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4" s="1">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E4" s="1">
         <v>3.75</v>
@@ -759,13 +747,13 @@
         <v>4</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H4" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -788,13 +776,13 @@
         <v>4</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -817,13 +805,13 @@
         <v>4</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>33</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -846,13 +834,13 @@
         <v>0</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="I7" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -866,7 +854,7 @@
         <v>4</v>
       </c>
       <c r="D8" s="1">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="E8" s="1">
         <v>4.5</v>
@@ -875,13 +863,13 @@
         <v>4</v>
       </c>
       <c r="G8" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>47</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -892,25 +880,25 @@
         <v>11</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D9" s="1">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E9" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="I9" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -921,28 +909,26 @@
         <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D10" s="1">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E10" s="1">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="F10" s="1">
         <v>4</v>
       </c>
       <c r="G10" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="H10" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I10" s="5"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
@@ -950,26 +936,14 @@
         <v>7</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="1">
-        <v>480</v>
-      </c>
-      <c r="E11" s="1">
-        <v>2</v>
-      </c>
-      <c r="F11" s="1">
-        <v>3.5</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>61</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="5"/>
     </row>
     <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
@@ -979,26 +953,14 @@
         <v>5</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="1">
-        <v>25</v>
-      </c>
-      <c r="E12" s="1">
-        <v>4</v>
-      </c>
-      <c r="F12" s="1">
-        <v>4</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>59</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
     </row>
     <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
@@ -1010,24 +972,12 @@
       <c r="C13" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="1">
-        <v>0</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0</v>
-      </c>
-      <c r="F13" s="1">
-        <v>0</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>64</v>
-      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
012: changes in the prompt design and crons were updated to include timezone in them.
</commit_message>
<xml_diff>
--- a/data/daily_routine.xlsx
+++ b/data/daily_routine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sai Swaroop\Desktop\Innvt\APPS\Routine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322E2A70-A642-4206-8BED-4A91E72A33D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70DD3560-F930-4AC5-A054-1F5D5656B87D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2DFCF397-A81A-4053-A0B6-07FE7B9B6438}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="66">
   <si>
     <t>23:40 – 07:00</t>
   </si>
@@ -105,13 +105,7 @@
     <t>Task</t>
   </si>
   <si>
-    <t>Time Block</t>
-  </si>
-  <si>
     <t>Win for day</t>
-  </si>
-  <si>
-    <t>Tomorrow's target</t>
   </si>
   <si>
     <t>Time spent (minutes)</t>
@@ -215,6 +209,28 @@
   <si>
     <t>wake 5mins up before time and 
 hydrate well</t>
+  </si>
+  <si>
+    <t>Time Block (IST time)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>went to play badminton for an hour for cardio
+ as it is holiday. Also did AI cource for sometime. Cooked and ate well</t>
+  </si>
+  <si>
+    <t>took rest</t>
+  </si>
+  <si>
+    <t>wasted time using mobile</t>
+  </si>
+  <si>
+    <t>to use the time well</t>
   </si>
 </sst>
 </file>
@@ -629,7 +645,7 @@
   <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.44140625" bestFit="1" customWidth="1"/>
@@ -642,7 +658,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>25</v>
@@ -651,22 +667,22 @@
         <v>24</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -674,7 +690,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>4</v>
@@ -689,13 +705,13 @@
         <v>3.5</v>
       </c>
       <c r="G2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>53</v>
-      </c>
       <c r="I2" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -703,10 +719,10 @@
         <v>23</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D3" s="1">
         <v>15</v>
@@ -718,13 +734,13 @@
         <v>3</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -747,13 +763,13 @@
         <v>4</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -776,13 +792,13 @@
         <v>4</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -805,13 +821,13 @@
         <v>4</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -834,13 +850,13 @@
         <v>0</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>42</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -863,13 +879,13 @@
         <v>4</v>
       </c>
       <c r="G8" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -892,13 +908,13 @@
         <v>0</v>
       </c>
       <c r="G9" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I9" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -921,14 +937,14 @@
         <v>4</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
@@ -936,13 +952,23 @@
         <v>7</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1">
+        <v>4</v>
+      </c>
+      <c r="F11" s="1">
+        <v>4</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>60</v>
+      </c>
       <c r="I11" s="5"/>
     </row>
     <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -953,13 +979,23 @@
         <v>5</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
+        <v>57</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>4</v>
+      </c>
+      <c r="F12" s="1">
+        <v>4</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>60</v>
+      </c>
       <c r="I12" s="5"/>
     </row>
     <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -972,12 +1008,24 @@
       <c r="C13" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
+      <c r="D13" s="1">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>65</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>